<commit_message>
chore(historico): atualizacao automatica 2026-10-01
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 01/09/2026  ·  Período coberto: 2024-08 a 2026-07  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 01/10/2026  ·  Período coberto: 2024-08 a 2026-09  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>101137</v>
+        <v>119385</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>138774</v>
+        <v>149651</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>61510</v>
+        <v>72752</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>95175</v>
+        <v>103283</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>58088</v>
+        <v>70119</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>38470</v>
+        <v>43438</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>33073</v>
+        <v>39367</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>29484</v>
+        <v>32866</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>31213</v>
+        <v>33563</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>89995</v>
+        <v>94738</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>20400</v>
+        <v>21936</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>57468</v>
+        <v>61358</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>11836</v>
+        <v>15703</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>10309</v>
+        <v>11475</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>8195</v>
+        <v>11633</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>8403</v>
+        <v>9261</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>56877</v>
+        <v>65906</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>82007</v>
+        <v>89079</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>33757</v>
+        <v>40068</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>56079</v>
+        <v>61280</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>1746</v>
+        <v>1904</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1532</v>
+        <v>1663</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>1079</v>
+        <v>1189</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1120</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>14209</v>
+        <v>15101</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8404</v>
+        <v>9016</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>9011</v>
+        <v>9610</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>6954</v>
+        <v>7424</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>28305</v>
+        <v>36474</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>46831</v>
+        <v>49893</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>18012</v>
+        <v>22312</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>32194</v>
+        <v>34604</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>43924</v>
+        <v>48187</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>48168</v>
+        <v>53744</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>33200</v>
+        <v>36325</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>40751</v>
+        <v>45269</v>
       </c>
     </row>
     <row r="16">
@@ -750,22 +750,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>145061</v>
+        <v>167572</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>186942</v>
+        <v>203395</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>94492</v>
+        <v>108822</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>135573</v>
+        <v>148146</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-08].</t>
+          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-09].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(dados): atualizacao com dump ENAP ate 2026-09
Roda o pipeline completo sobre o dump "ultimos 12 meses" (2025-10..2026-09):
historico publico, base fato do painel, pontes de publico/programa e as duas
distribuicoes pre-agregadas.

- Historico (Federal): +2026-08 e +2026-09; 2026-07 revisado de 6.105 para
  8.576 conclusoes (conclusoes tardias que o dump anterior ainda nao tinha).
  Total 158.493 conclusoes, 88.082 pessoas distintas.
- Base do painel (todas as esferas): 494.368 linhas, 26 meses (2024-08..2026-09),
  35/35 cursos com conclusao no periodo.
- Recorte do painel (IA/Dados): 370.967 conclusoes e 236.529 pessoas distintas,
  das quais 113.557 (31%) e 62.117 pessoas sao da esfera Federal.
- README e AGENTS.md: numeros da comparacao painel x historico publico
  atualizados juntos, como manda a nota de escopo.

PBIP regenerado com --csv-path absoluto: nenhum diff de estrutura, so os dados
que o modelo le do CSV mudaram.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/relatorio_capacitacao_ia.xlsx
+++ b/docs/relatorio_capacitacao_ia.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data: 01/09/2026  ·  Período coberto: 2024-08 a 2026-07  ·  Fonte: dadosaberto.evg.gov.br</t>
+          <t>Data: 16/10/2026  ·  Período coberto: 2024-08 a 2026-09  ·  Fonte: dadosaberto.evg.gov.br</t>
         </is>
       </c>
     </row>
@@ -557,16 +557,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>101137</v>
+        <v>119385</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>138774</v>
+        <v>149651</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>61510</v>
+        <v>72752</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>95175</v>
+        <v>103283</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>58088</v>
+        <v>70119</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>38470</v>
+        <v>43438</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>33073</v>
+        <v>39367</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>29484</v>
+        <v>32866</v>
       </c>
     </row>
     <row r="8">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>31213</v>
+        <v>33563</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>89995</v>
+        <v>94738</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>20400</v>
+        <v>21936</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>57468</v>
+        <v>61358</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>11836</v>
+        <v>15703</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>10309</v>
+        <v>11475</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>8195</v>
+        <v>11633</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>8403</v>
+        <v>9261</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>56877</v>
+        <v>65906</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>82007</v>
+        <v>89079</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>33757</v>
+        <v>40068</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>56079</v>
+        <v>61280</v>
       </c>
     </row>
     <row r="12">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>1746</v>
+        <v>1904</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1532</v>
+        <v>1663</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>1079</v>
+        <v>1189</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1120</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="13">
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>14209</v>
+        <v>15101</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8404</v>
+        <v>9016</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>9011</v>
+        <v>9610</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>6954</v>
+        <v>7424</v>
       </c>
     </row>
     <row r="14">
@@ -712,16 +712,16 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>28305</v>
+        <v>36474</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>46831</v>
+        <v>49893</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>18012</v>
+        <v>22312</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>32194</v>
+        <v>34604</v>
       </c>
     </row>
     <row r="15">
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>43924</v>
+        <v>48187</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>48168</v>
+        <v>53744</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>33200</v>
+        <v>36325</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>40751</v>
+        <v>45269</v>
       </c>
     </row>
     <row r="16">
@@ -750,22 +750,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>145061</v>
+        <v>167572</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>186942</v>
+        <v>203395</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>94492</v>
+        <v>108822</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>135573</v>
+        <v>148146</v>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-08].</t>
+          <t>Indicadores cobrem apenas IA e Dados (Gestão e Outros ficam de fora). Pessoas = contagem única de pessoas (codigo_pessoa); NÃO somam entre grupos. Matrículas = nº de conclusões (somam). Federal+Estadual+Municipal reconciliam o total público em matrículas; os poderes não (~32% dos registros públicos sem poder informado). "Setor Privado / não-servidor" agrega iniciativa privada, sociedade civil e público geral. Filtros: sit_matricula=Concluida; 35 cursos-alvo; dt_matricula em [2024-08, 2026-09].</t>
         </is>
       </c>
     </row>

</xml_diff>